<commit_message>
22-07-2026 all data updated
</commit_message>
<xml_diff>
--- a/module-4-excel-statistics/projects/coaching_management_app/coaching_revenue_generate_file.xlsx
+++ b/module-4-excel-statistics/projects/coaching_management_app/coaching_revenue_generate_file.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -650,16 +650,43 @@
         <v>46221.74738425926</v>
       </c>
     </row>
-    <row r="10">
-      <c r="F10" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>akash</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>130000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>46225.70320601852</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>total_sum</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="F11" t="n">
-        <v>190000</v>
+    <row r="12">
+      <c r="G12" t="n">
+        <v>245000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>